<commit_message>
feat(quotation): connect quotation import stops to customer-scoped canonical locations and separate pricing_basis from billing_type
</commit_message>
<xml_diff>
--- a/frontend/web-dashboard/public/templates/MERCON_August_Quotations_Import.xlsx
+++ b/frontend/web-dashboard/public/templates/MERCON_August_Quotations_Import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="98">
   <si>
     <t>Quotation Name</t>
   </si>
@@ -28,21 +28,21 @@
     <t>Vehicle Class</t>
   </si>
   <si>
-    <t>Line Type</t>
+    <t>Operation Type</t>
   </si>
   <si>
     <t>Pricing Basis</t>
   </si>
   <si>
+    <t>Billing Type</t>
+  </si>
+  <si>
     <t>Billing Rate (SAR)</t>
   </si>
   <si>
     <t>Driver Payout (SAR)</t>
   </si>
   <si>
-    <t>Trip Usage Count</t>
-  </si>
-  <si>
     <t>iMile — IMILE KHA to IMILE MUH (10 TON, Single Trip)</t>
   </si>
   <si>
@@ -61,6 +61,9 @@
     <t>Single Trip</t>
   </si>
   <si>
+    <t>Per Trip</t>
+  </si>
+  <si>
     <t>Monthly</t>
   </si>
   <si>
@@ -77,6 +80,9 @@
   </si>
   <si>
     <t>10 Hours Duty</t>
+  </si>
+  <si>
+    <t>Per Duty</t>
   </si>
   <si>
     <t>iMile — IMILE KHA to IMILE ABHA (10 TON, Single Trip)</t>
@@ -305,7 +311,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -313,13 +319,22 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3E3C3D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -334,8 +349,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -679,43 +697,43 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="10" width="18" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="8" width="15" customWidth="1"/>
+    <col min="9" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -741,28 +759,28 @@
       <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2">
         <v>499</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>50</v>
-      </c>
-      <c r="J2">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
@@ -773,51 +791,51 @@
       <c r="G3" t="s">
         <v>16</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3">
         <v>1750</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>149</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
         <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4">
         <v>430</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>60</v>
-      </c>
-      <c r="J4">
-        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -826,7 +844,7 @@
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
@@ -837,28 +855,28 @@
       <c r="G5" t="s">
         <v>16</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5">
         <v>450</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>60</v>
-      </c>
-      <c r="J5">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -869,31 +887,31 @@
       <c r="G6" t="s">
         <v>16</v>
       </c>
-      <c r="H6">
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6">
         <v>1050</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>64</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
         <v>15</v>
@@ -901,28 +919,28 @@
       <c r="G7" t="s">
         <v>16</v>
       </c>
-      <c r="H7">
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7">
         <v>966</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>105</v>
-      </c>
-      <c r="J7">
-        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -933,28 +951,28 @@
       <c r="G8" t="s">
         <v>16</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8">
         <v>581</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>50</v>
-      </c>
-      <c r="J8">
-        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
         <v>14</v>
@@ -965,31 +983,31 @@
       <c r="G9" t="s">
         <v>16</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9">
         <v>694</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>55</v>
-      </c>
-      <c r="J9">
-        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
         <v>37</v>
       </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" t="s">
-        <v>35</v>
-      </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
         <v>15</v>
@@ -997,28 +1015,28 @@
       <c r="G10" t="s">
         <v>16</v>
       </c>
-      <c r="H10">
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10">
         <v>530</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>50</v>
-      </c>
-      <c r="J10">
-        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
         <v>14</v>
@@ -1029,60 +1047,60 @@
       <c r="G11" t="s">
         <v>16</v>
       </c>
-      <c r="H11">
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11">
         <v>1737</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>190</v>
-      </c>
-      <c r="J11">
-        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
         <v>42</v>
       </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E12" t="s">
         <v>14</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G12" t="s">
         <v>16</v>
       </c>
-      <c r="H12">
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12">
         <v>387</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>60</v>
-      </c>
-      <c r="J12">
-        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
         <v>14</v>
@@ -1093,31 +1111,31 @@
       <c r="G13" t="s">
         <v>16</v>
       </c>
-      <c r="H13">
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13">
         <v>731</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>59</v>
-      </c>
-      <c r="J13">
-        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E14" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -1125,31 +1143,31 @@
       <c r="G14" t="s">
         <v>16</v>
       </c>
-      <c r="H14">
+      <c r="H14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14">
         <v>516</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>50</v>
-      </c>
-      <c r="J14">
-        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F15" t="s">
         <v>15</v>
@@ -1157,127 +1175,127 @@
       <c r="G15" t="s">
         <v>16</v>
       </c>
-      <c r="H15">
+      <c r="H15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15">
         <v>1500</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>149</v>
-      </c>
-      <c r="J15">
-        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" t="s">
         <v>52</v>
       </c>
-      <c r="B16" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" t="s">
-        <v>50</v>
-      </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G16" t="s">
         <v>16</v>
       </c>
-      <c r="H16">
+      <c r="H16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16">
         <v>1630</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>190</v>
-      </c>
-      <c r="J16">
-        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E17" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F17" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G17" t="s">
         <v>16</v>
       </c>
-      <c r="H17">
+      <c r="H17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17">
         <v>1630</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>200</v>
-      </c>
-      <c r="J17">
-        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E18" t="s">
         <v>14</v>
       </c>
       <c r="F18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>16</v>
-      </c>
-      <c r="H18">
+        <v>23</v>
+      </c>
+      <c r="H18" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18">
         <v>545</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>60</v>
-      </c>
-      <c r="J18">
-        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D19" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F19" t="s">
         <v>15</v>
@@ -1285,31 +1303,31 @@
       <c r="G19" t="s">
         <v>16</v>
       </c>
-      <c r="H19">
+      <c r="H19" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19">
         <v>370</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>35</v>
-      </c>
-      <c r="J19">
-        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E20" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
         <v>15</v>
@@ -1317,31 +1335,31 @@
       <c r="G20" t="s">
         <v>16</v>
       </c>
-      <c r="H20">
+      <c r="H20" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20">
         <v>966</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>105</v>
-      </c>
-      <c r="J20">
-        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F21" t="s">
         <v>15</v>
@@ -1349,28 +1367,28 @@
       <c r="G21" t="s">
         <v>16</v>
       </c>
-      <c r="H21">
+      <c r="H21" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21">
         <v>593</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>55</v>
-      </c>
-      <c r="J21">
-        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E22" t="s">
         <v>14</v>
@@ -1381,28 +1399,28 @@
       <c r="G22" t="s">
         <v>16</v>
       </c>
-      <c r="H22">
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22">
         <v>1665</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>144</v>
-      </c>
-      <c r="J22">
-        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E23" t="s">
         <v>14</v>
@@ -1413,31 +1431,31 @@
       <c r="G23" t="s">
         <v>16</v>
       </c>
-      <c r="H23">
+      <c r="H23" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23">
         <v>1150</v>
       </c>
-      <c r="I23">
+      <c r="J23">
         <v>64</v>
-      </c>
-      <c r="J23">
-        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E24" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F24" t="s">
         <v>15</v>
@@ -1445,28 +1463,28 @@
       <c r="G24" t="s">
         <v>16</v>
       </c>
-      <c r="H24">
+      <c r="H24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24">
         <v>1375</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>1200</v>
-      </c>
-      <c r="J24">
-        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" t="s">
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s">
         <v>14</v>
@@ -1477,31 +1495,31 @@
       <c r="G25" t="s">
         <v>16</v>
       </c>
-      <c r="H25">
+      <c r="H25" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25">
         <v>2090</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>149</v>
-      </c>
-      <c r="J25">
-        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C26" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E26" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F26" t="s">
         <v>15</v>
@@ -1509,31 +1527,31 @@
       <c r="G26" t="s">
         <v>16</v>
       </c>
-      <c r="H26">
+      <c r="H26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26">
         <v>850</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>124</v>
-      </c>
-      <c r="J26">
-        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E27" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F27" t="s">
         <v>15</v>
@@ -1541,28 +1559,28 @@
       <c r="G27" t="s">
         <v>16</v>
       </c>
-      <c r="H27">
+      <c r="H27" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27">
         <v>850</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>1000</v>
-      </c>
-      <c r="J27">
-        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D28" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E28" t="s">
         <v>14</v>
@@ -1573,31 +1591,31 @@
       <c r="G28" t="s">
         <v>16</v>
       </c>
-      <c r="H28">
+      <c r="H28" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28">
         <v>983</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>64</v>
-      </c>
-      <c r="J28">
-        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D29" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E29" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F29" t="s">
         <v>15</v>
@@ -1605,31 +1623,31 @@
       <c r="G29" t="s">
         <v>16</v>
       </c>
-      <c r="H29">
+      <c r="H29" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29">
         <v>850</v>
       </c>
-      <c r="I29">
+      <c r="J29">
         <v>950</v>
-      </c>
-      <c r="J29">
-        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E30" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F30" t="s">
         <v>15</v>
@@ -1637,31 +1655,31 @@
       <c r="G30" t="s">
         <v>16</v>
       </c>
-      <c r="H30">
+      <c r="H30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30">
         <v>900</v>
       </c>
-      <c r="I30">
+      <c r="J30">
         <v>1250</v>
-      </c>
-      <c r="J30">
-        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E31" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F31" t="s">
         <v>15</v>
@@ -1669,28 +1687,28 @@
       <c r="G31" t="s">
         <v>16</v>
       </c>
-      <c r="H31">
+      <c r="H31" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31">
         <v>1300</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>1650</v>
-      </c>
-      <c r="J31">
-        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B32" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D32" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E32" t="s">
         <v>14</v>
@@ -1701,31 +1719,31 @@
       <c r="G32" t="s">
         <v>16</v>
       </c>
-      <c r="H32">
+      <c r="H32" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32">
         <v>450</v>
       </c>
-      <c r="I32">
+      <c r="J32">
         <v>185</v>
-      </c>
-      <c r="J32">
-        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B33" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C33" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D33" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E33" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F33" t="s">
         <v>15</v>
@@ -1733,31 +1751,31 @@
       <c r="G33" t="s">
         <v>16</v>
       </c>
-      <c r="H33">
+      <c r="H33" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33">
         <v>1375</v>
       </c>
-      <c r="I33">
+      <c r="J33">
         <v>1200</v>
-      </c>
-      <c r="J33">
-        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E34" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F34" t="s">
         <v>15</v>
@@ -1765,31 +1783,31 @@
       <c r="G34" t="s">
         <v>16</v>
       </c>
-      <c r="H34">
+      <c r="H34" t="s">
+        <v>17</v>
+      </c>
+      <c r="I34">
         <v>900</v>
       </c>
-      <c r="I34">
+      <c r="J34">
         <v>140</v>
-      </c>
-      <c r="J34">
-        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E35" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F35" t="s">
         <v>15</v>
@@ -1797,31 +1815,31 @@
       <c r="G35" t="s">
         <v>16</v>
       </c>
-      <c r="H35">
+      <c r="H35" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35">
         <v>375</v>
       </c>
-      <c r="I35">
+      <c r="J35">
         <v>400</v>
-      </c>
-      <c r="J35">
-        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E36" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F36" t="s">
         <v>15</v>
@@ -1829,28 +1847,28 @@
       <c r="G36" t="s">
         <v>16</v>
       </c>
-      <c r="H36">
+      <c r="H36" t="s">
+        <v>17</v>
+      </c>
+      <c r="I36">
         <v>375</v>
       </c>
-      <c r="I36">
+      <c r="J36">
         <v>300</v>
-      </c>
-      <c r="J36">
-        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" t="s">
         <v>11</v>
       </c>
       <c r="C37" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D37" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E37" t="s">
         <v>14</v>
@@ -1861,28 +1879,28 @@
       <c r="G37" t="s">
         <v>16</v>
       </c>
-      <c r="H37">
+      <c r="H37" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37">
         <v>490</v>
       </c>
-      <c r="I37">
+      <c r="J37">
         <v>35</v>
-      </c>
-      <c r="J37">
-        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" t="s">
         <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
         <v>14</v>
@@ -1893,28 +1911,28 @@
       <c r="G38" t="s">
         <v>16</v>
       </c>
-      <c r="H38">
+      <c r="H38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38">
         <v>1015</v>
       </c>
-      <c r="I38">
+      <c r="J38">
         <v>64</v>
-      </c>
-      <c r="J38">
-        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C39" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D39" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E39" t="s">
         <v>14</v>
@@ -1925,31 +1943,31 @@
       <c r="G39" t="s">
         <v>16</v>
       </c>
-      <c r="H39">
+      <c r="H39" t="s">
+        <v>17</v>
+      </c>
+      <c r="I39">
         <v>1737</v>
       </c>
-      <c r="I39">
+      <c r="J39">
         <v>130</v>
-      </c>
-      <c r="J39">
-        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E40" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F40" t="s">
         <v>15</v>
@@ -1957,60 +1975,60 @@
       <c r="G40" t="s">
         <v>16</v>
       </c>
-      <c r="H40">
+      <c r="H40" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40">
         <v>2250</v>
       </c>
-      <c r="I40">
+      <c r="J40">
         <v>280</v>
-      </c>
-      <c r="J40">
-        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" t="s">
+        <v>29</v>
+      </c>
+      <c r="C41" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E41" t="s">
+        <v>32</v>
+      </c>
+      <c r="F41" t="s">
+        <v>15</v>
+      </c>
+      <c r="G41" t="s">
+        <v>16</v>
+      </c>
+      <c r="H41" t="s">
+        <v>17</v>
+      </c>
+      <c r="I41">
+        <v>593</v>
+      </c>
+      <c r="J41">
         <v>59</v>
-      </c>
-      <c r="B41" t="s">
-        <v>27</v>
-      </c>
-      <c r="C41" t="s">
-        <v>35</v>
-      </c>
-      <c r="D41" t="s">
-        <v>60</v>
-      </c>
-      <c r="E41" t="s">
-        <v>30</v>
-      </c>
-      <c r="F41" t="s">
-        <v>15</v>
-      </c>
-      <c r="G41" t="s">
-        <v>16</v>
-      </c>
-      <c r="H41">
-        <v>593</v>
-      </c>
-      <c r="I41">
-        <v>59</v>
-      </c>
-      <c r="J41">
-        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E42" t="s">
         <v>14</v>
@@ -2021,31 +2039,31 @@
       <c r="G42" t="s">
         <v>16</v>
       </c>
-      <c r="H42">
+      <c r="H42" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42">
         <v>500</v>
       </c>
-      <c r="I42">
+      <c r="J42">
         <v>45</v>
-      </c>
-      <c r="J42">
-        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B43" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C43" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D43" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E43" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F43" t="s">
         <v>15</v>
@@ -2053,28 +2071,28 @@
       <c r="G43" t="s">
         <v>16</v>
       </c>
-      <c r="H43">
+      <c r="H43" t="s">
+        <v>17</v>
+      </c>
+      <c r="I43">
         <v>593</v>
       </c>
-      <c r="I43">
+      <c r="J43">
         <v>1000</v>
-      </c>
-      <c r="J43">
-        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" t="s">
         <v>11</v>
       </c>
       <c r="C44" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D44" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E44" t="s">
         <v>14</v>
@@ -2085,14 +2103,14 @@
       <c r="G44" t="s">
         <v>16</v>
       </c>
-      <c r="H44">
+      <c r="H44" t="s">
+        <v>17</v>
+      </c>
+      <c r="I44">
         <v>1015</v>
       </c>
-      <c r="I44">
+      <c r="J44">
         <v>64</v>
-      </c>
-      <c r="J44">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>